<commit_message>
shablonlar: guruh_kodi va kategoriya_kodi uchun izoh
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/clients-shablon.xlsx
+++ b/docs/templates/clients-shablon.xlsx
@@ -8,6 +8,23 @@
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
+    <comment ref="C2" authorId="0">
+      <text>
+        <r>
+          <t>avval /client-categories orqali yaratiladi</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -440,5 +457,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
shablonlar: buxgalter uchun yo'riqnoma va tuzatishlar
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/clients-shablon.xlsx
+++ b/docs/templates/clients-shablon.xlsx
@@ -5,6 +5,7 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Import" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Yo'riqnoma" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -19,7 +20,7 @@
     <comment ref="C2" authorId="0">
       <text>
         <r>
-          <t>avval /client-categories orqali yaratiladi</t>
+          <t>Bu mijoz kategoriyasi avval tizimda yaratilgan bo'lishi kerak (Ma'lumotnomalar → Mijoz kategoriyalari)</t>
         </r>
       </text>
     </comment>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
   <si>
     <t>mijoz_kodi</t>
   </si>
@@ -46,6 +47,39 @@
   </si>
   <si>
     <t>K001</t>
+  </si>
+  <si>
+    <t>ustun</t>
+  </si>
+  <si>
+    <t>majburiymi</t>
+  </si>
+  <si>
+    <t>format</t>
+  </si>
+  <si>
+    <t>misol</t>
+  </si>
+  <si>
+    <t>Ha</t>
+  </si>
+  <si>
+    <t>Matn, ko'pi bilan 50 belgi</t>
+  </si>
+  <si>
+    <t>Matn, ko'pi bilan 200 belgi</t>
+  </si>
+  <si>
+    <t>Yo'q</t>
+  </si>
+  <si>
+    <t>Mijoz kategoriyasi kodi (Ma'lumotnomalar → Mijoz kategoriyalari)</t>
+  </si>
+  <si>
+    <t>2-qatordagi namuna — faqat ko'rsatma. Uni o'chirib, o'z ma'lumotingizni yozing, aks holda namuna ham import qilinadi.</t>
+  </si>
+  <si>
+    <t>1-qator (sarlavha) o'zgarmasligi kerak. Import faqat shu faylning birinchi varag'ini o'qiydi — «Yo'riqnoma» varag'i hisobga olinmaydi.</t>
   </si>
 </sst>
 </file>
@@ -84,9 +118,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -429,7 +469,9 @@
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="3" width="20" customWidth="1"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -459,4 +501,87 @@
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="3" max="3" width="67" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
shablonlar: namuna qatorsiz (faqat sarlavha + Yo'riqnoma), test sanalari 2026
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/clients-shablon.xlsx
+++ b/docs/templates/clients-shablon.xlsx
@@ -17,7 +17,7 @@
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="C2" authorId="0">
+    <comment ref="C1" authorId="0">
       <text>
         <r>
           <t>Bu mijoz kategoriyasi avval tizimda yaratilgan bo'lishi kerak (Ma'lumotnomalar → Mijoz kategoriyalari)</t>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>mijoz_kodi</t>
   </si>
@@ -40,43 +40,43 @@
     <t>kategoriya_kodi</t>
   </si>
   <si>
+    <t>ustun</t>
+  </si>
+  <si>
+    <t>majburiymi</t>
+  </si>
+  <si>
+    <t>format</t>
+  </si>
+  <si>
+    <t>misol</t>
+  </si>
+  <si>
+    <t>Ha</t>
+  </si>
+  <si>
+    <t>Matn, ko'pi bilan 50 belgi</t>
+  </si>
+  <si>
     <t>C001</t>
   </si>
   <si>
+    <t>Matn, ko'pi bilan 200 belgi</t>
+  </si>
+  <si>
     <t>Namuna mijoz</t>
   </si>
   <si>
+    <t>Yo'q</t>
+  </si>
+  <si>
+    <t>Mijoz kategoriyasi kodi (Ma'lumotnomalar → Mijoz kategoriyalari)</t>
+  </si>
+  <si>
     <t>K001</t>
   </si>
   <si>
-    <t>ustun</t>
-  </si>
-  <si>
-    <t>majburiymi</t>
-  </si>
-  <si>
-    <t>format</t>
-  </si>
-  <si>
-    <t>misol</t>
-  </si>
-  <si>
-    <t>Ha</t>
-  </si>
-  <si>
-    <t>Matn, ko'pi bilan 50 belgi</t>
-  </si>
-  <si>
-    <t>Matn, ko'pi bilan 200 belgi</t>
-  </si>
-  <si>
-    <t>Yo'q</t>
-  </si>
-  <si>
-    <t>Mijoz kategoriyasi kodi (Ma'lumotnomalar → Mijoz kategoriyalari)</t>
-  </si>
-  <si>
-    <t>2-qatordagi namuna — faqat ko'rsatma. Uni o'chirib, o'z ma'lumotingizni yozing, aks holda namuna ham import qilinadi.</t>
+    <t>«misol» ustunidagi qiymatlar — faqat ko'rsatma. 1-varaqning 2-qatoridan boshlab o'z ma'lumotingizni yozing.</t>
   </si>
   <si>
     <t>1-qator (sarlavha) o'zgarmasligi kerak. Import faqat shu faylning birinchi varag'ini o'qiydi — «Yo'riqnoma» varag'i hisobga olinmaydi.</t>
@@ -466,11 +466,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="2" max="2" width="7" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
   </cols>
   <sheetData>
@@ -483,17 +483,6 @@
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -516,16 +505,16 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -533,13 +522,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -547,13 +536,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="D3" s="3" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -561,13 +550,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>